<commit_message>
Update metadata for 1.2.1 and 1.2.2
</commit_message>
<xml_diff>
--- a/data/2025_RW-SDG_Data.xlsx
+++ b/data/2025_RW-SDG_Data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\GGessienne\Documents\sdg-data-rwanda\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9050FAF0-A523-4F93-9C5B-8D4BAE569DB6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1A35F557-FEDC-4CCB-A562-0BED45EA2C6E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-90" yWindow="-90" windowWidth="19380" windowHeight="10260" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -3362,10 +3362,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="3">
+  <numFmts count="4">
     <numFmt numFmtId="164" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
     <numFmt numFmtId="165" formatCode="_-* #,##0.00\ _€_-;\-* #,##0.00\ _€_-;_-* &quot;-&quot;??\ _€_-;_-@_-"/>
     <numFmt numFmtId="166" formatCode="0.0"/>
+    <numFmt numFmtId="167" formatCode="0.000"/>
   </numFmts>
   <fonts count="13" x14ac:knownFonts="1">
     <font>
@@ -3489,7 +3490,7 @@
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="2"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -3499,6 +3500,8 @@
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="2" applyFont="1"/>
     <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="10">
     <cellStyle name="Bad" xfId="1" builtinId="27"/>
@@ -13806,28 +13809,28 @@
       <c r="T45" t="s">
         <v>89</v>
       </c>
-      <c r="AA45" s="7">
+      <c r="AA45" s="10">
         <v>0.443</v>
       </c>
-      <c r="AF45" s="7">
+      <c r="AF45" s="9">
         <v>0.35</v>
       </c>
-      <c r="AG45" s="7">
+      <c r="AG45" s="9">
         <v>0.24</v>
       </c>
-      <c r="AH45" s="7">
+      <c r="AH45" s="10">
         <v>0.16700000000000001</v>
       </c>
-      <c r="AJ45" s="7">
+      <c r="AJ45" s="9">
         <v>0.17</v>
       </c>
-      <c r="AM45" s="7">
+      <c r="AM45" s="9">
         <v>0.15</v>
       </c>
-      <c r="AR45" s="7">
+      <c r="AR45" s="10">
         <v>0.129</v>
       </c>
-      <c r="AT45" s="7">
+      <c r="AT45" s="10">
         <v>0.13600000000000001</v>
       </c>
     </row>
@@ -13874,22 +13877,22 @@
       <c r="T46" t="s">
         <v>89</v>
       </c>
-      <c r="AG46" s="7">
+      <c r="AG46" s="9">
         <v>0.09</v>
       </c>
-      <c r="AH46" s="7">
+      <c r="AH46" s="10">
         <v>6.5000000000000002E-2</v>
       </c>
-      <c r="AJ46" s="7">
+      <c r="AJ46" s="9">
         <v>7.0000000000000007E-2</v>
       </c>
-      <c r="AM46" s="7">
+      <c r="AM46" s="9">
         <v>7.0000000000000007E-2</v>
       </c>
-      <c r="AR46" s="7">
+      <c r="AR46" s="10">
         <v>5.6000000000000001E-2</v>
       </c>
-      <c r="AT46" s="7">
+      <c r="AT46" s="10">
         <v>6.5000000000000002E-2</v>
       </c>
     </row>
@@ -13936,22 +13939,22 @@
       <c r="T47" t="s">
         <v>89</v>
       </c>
-      <c r="AG47" s="7">
+      <c r="AG47" s="9">
         <v>0.27</v>
       </c>
-      <c r="AH47" s="7">
+      <c r="AH47" s="10">
         <v>0.187</v>
       </c>
-      <c r="AJ47" s="7">
+      <c r="AJ47" s="9">
         <v>0.19</v>
       </c>
-      <c r="AM47" s="7">
+      <c r="AM47" s="9">
         <v>0.17</v>
       </c>
-      <c r="AR47" s="7">
+      <c r="AR47" s="10">
         <v>0.159</v>
       </c>
-      <c r="AT47" s="7">
+      <c r="AT47" s="10">
         <v>0.16400000000000001</v>
       </c>
     </row>
@@ -13998,22 +14001,22 @@
       <c r="T48" t="s">
         <v>89</v>
       </c>
-      <c r="AG48" s="7">
+      <c r="AG48" s="9">
         <v>0.12</v>
       </c>
-      <c r="AH48" s="7">
+      <c r="AH48" s="10">
         <v>6.4000000000000001E-2</v>
       </c>
-      <c r="AJ48" s="7">
+      <c r="AJ48" s="9">
         <v>7.0000000000000007E-2</v>
       </c>
-      <c r="AM48" s="7">
+      <c r="AM48" s="9">
         <v>7.0000000000000007E-2</v>
       </c>
-      <c r="AR48" s="7">
+      <c r="AR48" s="10">
         <v>0.04</v>
       </c>
-      <c r="AT48" s="7">
+      <c r="AT48" s="10">
         <v>5.2999999999999999E-2</v>
       </c>
     </row>
@@ -14060,22 +14063,22 @@
       <c r="T49" t="s">
         <v>89</v>
       </c>
-      <c r="AG49" s="7">
+      <c r="AG49" s="9">
         <v>0.28999999999999998</v>
       </c>
-      <c r="AH49" s="7">
+      <c r="AH49" s="10">
         <v>0.17100000000000001</v>
       </c>
-      <c r="AJ49" s="7">
+      <c r="AJ49" s="9">
         <v>0.21</v>
       </c>
-      <c r="AM49" s="7">
+      <c r="AM49" s="9">
         <v>0.19</v>
       </c>
-      <c r="AR49" s="7">
+      <c r="AR49" s="10">
         <v>0.14899999999999999</v>
       </c>
-      <c r="AT49" s="7">
+      <c r="AT49" s="10">
         <v>0.158</v>
       </c>
     </row>
@@ -14122,22 +14125,22 @@
       <c r="T50" t="s">
         <v>89</v>
       </c>
-      <c r="AG50" s="7">
+      <c r="AG50" s="9">
         <v>0.25</v>
       </c>
-      <c r="AH50" s="7">
+      <c r="AH50" s="10">
         <v>0.189</v>
       </c>
-      <c r="AJ50" s="7">
+      <c r="AJ50" s="9">
         <v>0.19</v>
       </c>
-      <c r="AM50" s="7">
+      <c r="AM50" s="9">
         <v>0.16</v>
       </c>
-      <c r="AR50" s="7">
+      <c r="AR50" s="10">
         <v>0.15</v>
       </c>
-      <c r="AT50" s="7">
+      <c r="AT50" s="10">
         <v>0.14899999999999999</v>
       </c>
     </row>
@@ -14184,22 +14187,22 @@
       <c r="T51" t="s">
         <v>89</v>
       </c>
-      <c r="AG51" s="7">
+      <c r="AG51" s="9">
         <v>0.18</v>
       </c>
-      <c r="AH51" s="7">
+      <c r="AH51" s="10">
         <v>0.161</v>
       </c>
-      <c r="AJ51" s="7">
+      <c r="AJ51" s="9">
         <v>0.14000000000000001</v>
       </c>
-      <c r="AM51" s="7">
+      <c r="AM51" s="9">
         <v>0.11</v>
       </c>
-      <c r="AR51" s="7">
+      <c r="AR51" s="10">
         <v>0.122</v>
       </c>
-      <c r="AT51" s="7">
+      <c r="AT51" s="10">
         <v>0.123</v>
       </c>
     </row>
@@ -14246,22 +14249,22 @@
       <c r="T52" t="s">
         <v>89</v>
       </c>
-      <c r="AG52" s="7">
+      <c r="AG52" s="9">
         <v>0.26</v>
       </c>
-      <c r="AH52" s="7">
+      <c r="AH52" s="10">
         <v>0.192</v>
       </c>
-      <c r="AJ52" s="7">
+      <c r="AJ52" s="9">
         <v>0.18</v>
       </c>
-      <c r="AM52" s="7">
+      <c r="AM52" s="9">
         <v>0.17</v>
       </c>
-      <c r="AR52" s="7">
+      <c r="AR52" s="10">
         <v>0.15</v>
       </c>
-      <c r="AT52" s="7">
+      <c r="AT52" s="10">
         <v>0.157</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Update Indicators 1.5.1 - 1.5.4
</commit_message>
<xml_diff>
--- a/data/2025_RW-SDG_Data.xlsx
+++ b/data/2025_RW-SDG_Data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\GGessienne\Documents\sdg-data-rwanda\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{200B5422-8A4E-4CAB-8252-D9ECAB22E1DF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{66BD56BF-2C8F-4FB6-A82D-ABD1769F3C8C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-90" yWindow="-90" windowWidth="19380" windowHeight="10260" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -48,7 +48,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7966" uniqueCount="1077">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7966" uniqueCount="1092">
   <si>
     <t>Indicator</t>
   </si>
@@ -3357,6 +3357,51 @@
   </si>
   <si>
     <t>Percentage of farmers with the right to sell or use land as collateral</t>
+  </si>
+  <si>
+    <t>Direct economic loss attributed to disasters in relation to global gross domestic product (GDP)</t>
+  </si>
+  <si>
+    <t>Houses damaged by disaster</t>
+  </si>
+  <si>
+    <t>Ha of crops damaged by disaster</t>
+  </si>
+  <si>
+    <t>Classrooms damaged by disaster</t>
+  </si>
+  <si>
+    <t>Health centers damaged by disaster</t>
+  </si>
+  <si>
+    <t>Bridges damaged by disaster</t>
+  </si>
+  <si>
+    <t>Administrative offices damaged by disaster</t>
+  </si>
+  <si>
+    <t>Transmission lines damaged by disaster</t>
+  </si>
+  <si>
+    <t>Water supply structures damaged by disaster</t>
+  </si>
+  <si>
+    <t>Markets damaged by disaster</t>
+  </si>
+  <si>
+    <t>Factories damaged by disaster</t>
+  </si>
+  <si>
+    <t>Ha of forests damaged by disaster</t>
+  </si>
+  <si>
+    <t>Churches damaged by disaster</t>
+  </si>
+  <si>
+    <t>Road sections damaged by disaster</t>
+  </si>
+  <si>
+    <t>Cattle and livestock lost due to disaster</t>
   </si>
 </sst>
 </file>
@@ -15468,7 +15513,7 @@
         <v>854</v>
       </c>
       <c r="B73" t="s">
-        <v>853</v>
+        <v>1077</v>
       </c>
       <c r="C73" t="s">
         <v>865</v>
@@ -15495,7 +15540,7 @@
         <v>886</v>
       </c>
       <c r="P73" t="s">
-        <v>912</v>
+        <v>1078</v>
       </c>
       <c r="R73" t="s">
         <v>89</v>
@@ -15530,7 +15575,7 @@
         <v>854</v>
       </c>
       <c r="B74" t="s">
-        <v>853</v>
+        <v>1077</v>
       </c>
       <c r="C74" t="s">
         <v>869</v>
@@ -15557,7 +15602,7 @@
         <v>886</v>
       </c>
       <c r="P74" t="s">
-        <v>855</v>
+        <v>1079</v>
       </c>
       <c r="R74" t="s">
         <v>89</v>
@@ -15592,7 +15637,7 @@
         <v>854</v>
       </c>
       <c r="B75" t="s">
-        <v>853</v>
+        <v>1077</v>
       </c>
       <c r="C75" t="s">
         <v>867</v>
@@ -15619,7 +15664,7 @@
         <v>886</v>
       </c>
       <c r="P75" t="s">
-        <v>856</v>
+        <v>1080</v>
       </c>
       <c r="R75" t="s">
         <v>89</v>
@@ -15654,7 +15699,7 @@
         <v>854</v>
       </c>
       <c r="B76" t="s">
-        <v>853</v>
+        <v>1077</v>
       </c>
       <c r="C76" t="s">
         <v>871</v>
@@ -15681,7 +15726,7 @@
         <v>886</v>
       </c>
       <c r="P76" t="s">
-        <v>857</v>
+        <v>1081</v>
       </c>
       <c r="R76" t="s">
         <v>89</v>
@@ -15716,7 +15761,7 @@
         <v>854</v>
       </c>
       <c r="B77" t="s">
-        <v>853</v>
+        <v>1077</v>
       </c>
       <c r="C77" t="s">
         <v>868</v>
@@ -15743,7 +15788,7 @@
         <v>886</v>
       </c>
       <c r="P77" t="s">
-        <v>858</v>
+        <v>1082</v>
       </c>
       <c r="R77" t="s">
         <v>89</v>
@@ -15778,7 +15823,7 @@
         <v>854</v>
       </c>
       <c r="B78" t="s">
-        <v>853</v>
+        <v>1077</v>
       </c>
       <c r="C78" t="s">
         <v>872</v>
@@ -15805,7 +15850,7 @@
         <v>886</v>
       </c>
       <c r="P78" t="s">
-        <v>859</v>
+        <v>1083</v>
       </c>
       <c r="R78" t="s">
         <v>89</v>
@@ -15840,7 +15885,7 @@
         <v>854</v>
       </c>
       <c r="B79" t="s">
-        <v>853</v>
+        <v>1077</v>
       </c>
       <c r="C79" t="s">
         <v>866</v>
@@ -15867,7 +15912,7 @@
         <v>886</v>
       </c>
       <c r="P79" t="s">
-        <v>860</v>
+        <v>1084</v>
       </c>
       <c r="R79" t="s">
         <v>89</v>
@@ -15902,7 +15947,7 @@
         <v>854</v>
       </c>
       <c r="B80" t="s">
-        <v>853</v>
+        <v>1077</v>
       </c>
       <c r="C80" t="s">
         <v>870</v>
@@ -15929,7 +15974,7 @@
         <v>886</v>
       </c>
       <c r="P80" t="s">
-        <v>861</v>
+        <v>1085</v>
       </c>
       <c r="R80" t="s">
         <v>89</v>
@@ -15964,7 +16009,7 @@
         <v>854</v>
       </c>
       <c r="B81" t="s">
-        <v>853</v>
+        <v>1077</v>
       </c>
       <c r="C81" t="s">
         <v>873</v>
@@ -15991,7 +16036,7 @@
         <v>886</v>
       </c>
       <c r="P81" t="s">
-        <v>862</v>
+        <v>1086</v>
       </c>
       <c r="R81" t="s">
         <v>89</v>
@@ -16023,7 +16068,7 @@
         <v>854</v>
       </c>
       <c r="B82" t="s">
-        <v>853</v>
+        <v>1077</v>
       </c>
       <c r="C82" t="s">
         <v>874</v>
@@ -16050,7 +16095,7 @@
         <v>886</v>
       </c>
       <c r="P82" t="s">
-        <v>863</v>
+        <v>1087</v>
       </c>
       <c r="R82" t="s">
         <v>89</v>
@@ -16082,7 +16127,7 @@
         <v>854</v>
       </c>
       <c r="B83" t="s">
-        <v>853</v>
+        <v>1077</v>
       </c>
       <c r="C83" t="s">
         <v>875</v>
@@ -16109,7 +16154,7 @@
         <v>886</v>
       </c>
       <c r="P83" t="s">
-        <v>864</v>
+        <v>1088</v>
       </c>
       <c r="R83" t="s">
         <v>89</v>
@@ -16138,7 +16183,7 @@
         <v>854</v>
       </c>
       <c r="B84" t="s">
-        <v>853</v>
+        <v>1077</v>
       </c>
       <c r="C84" t="s">
         <v>883</v>
@@ -16165,7 +16210,7 @@
         <v>886</v>
       </c>
       <c r="P84" t="s">
-        <v>881</v>
+        <v>1089</v>
       </c>
       <c r="R84" t="s">
         <v>89</v>
@@ -16197,7 +16242,7 @@
         <v>854</v>
       </c>
       <c r="B85" t="s">
-        <v>853</v>
+        <v>1077</v>
       </c>
       <c r="C85" t="s">
         <v>884</v>
@@ -16224,7 +16269,7 @@
         <v>886</v>
       </c>
       <c r="P85" t="s">
-        <v>913</v>
+        <v>1090</v>
       </c>
       <c r="R85" t="s">
         <v>89</v>
@@ -16256,7 +16301,7 @@
         <v>854</v>
       </c>
       <c r="B86" t="s">
-        <v>853</v>
+        <v>1077</v>
       </c>
       <c r="C86" t="s">
         <v>885</v>
@@ -16283,7 +16328,7 @@
         <v>886</v>
       </c>
       <c r="P86" t="s">
-        <v>882</v>
+        <v>1091</v>
       </c>
       <c r="R86" t="s">
         <v>89</v>
@@ -16350,10 +16395,10 @@
       <c r="T87" t="s">
         <v>89</v>
       </c>
+      <c r="AJ87">
+        <v>73.3</v>
+      </c>
       <c r="AM87">
-        <v>77.3</v>
-      </c>
-      <c r="AN87">
         <v>96.7</v>
       </c>
       <c r="AO87">
@@ -16369,6 +16414,9 @@
         <v>100</v>
       </c>
       <c r="AS87">
+        <v>100</v>
+      </c>
+      <c r="AT87">
         <v>100</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Add 2025 and 2026 columns; fill in for 1.a.2
</commit_message>
<xml_diff>
--- a/data/2025_RW-SDG_Data.xlsx
+++ b/data/2025_RW-SDG_Data.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\GGessienne\Documents\sdg-data-rwanda\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9B54F145-B73F-431E-8B6B-5AEE4CD57B4C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{50C72346-FE13-423F-A1B3-986E79831C49}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-90" yWindow="-90" windowWidth="19380" windowHeight="10260" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -11256,7 +11256,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AU581"/>
+  <dimension ref="A1:AV581"/>
   <sheetFormatPr defaultColWidth="9.1796875" defaultRowHeight="20" customHeight="1" x14ac:dyDescent="0.75"/>
   <cols>
     <col min="1" max="1" width="10.6328125" customWidth="1"/>
@@ -11266,7 +11266,7 @@
     <col min="22" max="46" width="9.08984375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:46" ht="20" customHeight="1" x14ac:dyDescent="0.75">
+    <row r="1" spans="1:48" ht="20" customHeight="1" x14ac:dyDescent="0.75">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -11405,8 +11405,14 @@
       <c r="AT1" s="2">
         <v>2024</v>
       </c>
-    </row>
-    <row r="2" spans="1:46" ht="20" customHeight="1" x14ac:dyDescent="0.75">
+      <c r="AU1" s="2">
+        <v>2025</v>
+      </c>
+      <c r="AV1" s="2">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="2" spans="1:48" ht="20" customHeight="1" x14ac:dyDescent="0.75">
       <c r="A2" t="s">
         <v>121</v>
       </c>
@@ -11466,7 +11472,7 @@
         <v>38.6</v>
       </c>
     </row>
-    <row r="3" spans="1:46" ht="20" customHeight="1" x14ac:dyDescent="0.75">
+    <row r="3" spans="1:48" ht="20" customHeight="1" x14ac:dyDescent="0.75">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -11525,7 +11531,7 @@
         <v>27.4</v>
       </c>
     </row>
-    <row r="4" spans="1:46" ht="20" customHeight="1" x14ac:dyDescent="0.75">
+    <row r="4" spans="1:48" ht="20" customHeight="1" x14ac:dyDescent="0.75">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -11581,7 +11587,7 @@
         <v>24.9</v>
       </c>
     </row>
-    <row r="5" spans="1:46" ht="20" customHeight="1" x14ac:dyDescent="0.75">
+    <row r="5" spans="1:48" ht="20" customHeight="1" x14ac:dyDescent="0.75">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -11637,7 +11643,7 @@
         <v>25.4</v>
       </c>
     </row>
-    <row r="6" spans="1:46" ht="20" customHeight="1" x14ac:dyDescent="0.75">
+    <row r="6" spans="1:48" ht="20" customHeight="1" x14ac:dyDescent="0.75">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -11693,7 +11699,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="7" spans="1:46" ht="20" customHeight="1" x14ac:dyDescent="0.75">
+    <row r="7" spans="1:48" ht="20" customHeight="1" x14ac:dyDescent="0.75">
       <c r="A7" t="s">
         <v>9</v>
       </c>
@@ -11749,7 +11755,7 @@
         <v>29.9</v>
       </c>
     </row>
-    <row r="8" spans="1:46" ht="20" customHeight="1" x14ac:dyDescent="0.75">
+    <row r="8" spans="1:48" ht="20" customHeight="1" x14ac:dyDescent="0.75">
       <c r="A8" t="s">
         <v>9</v>
       </c>
@@ -11808,7 +11814,7 @@
         <v>16.7</v>
       </c>
     </row>
-    <row r="9" spans="1:46" ht="20" customHeight="1" x14ac:dyDescent="0.75">
+    <row r="9" spans="1:48" ht="20" customHeight="1" x14ac:dyDescent="0.75">
       <c r="A9" t="s">
         <v>9</v>
       </c>
@@ -11867,7 +11873,7 @@
         <v>31.6</v>
       </c>
     </row>
-    <row r="10" spans="1:46" ht="20" customHeight="1" x14ac:dyDescent="0.75">
+    <row r="10" spans="1:48" ht="20" customHeight="1" x14ac:dyDescent="0.75">
       <c r="A10" t="s">
         <v>9</v>
       </c>
@@ -11929,7 +11935,7 @@
         <v>9.1</v>
       </c>
     </row>
-    <row r="11" spans="1:46" ht="20" customHeight="1" x14ac:dyDescent="0.75">
+    <row r="11" spans="1:48" ht="20" customHeight="1" x14ac:dyDescent="0.75">
       <c r="A11" t="s">
         <v>9</v>
       </c>
@@ -11991,7 +11997,7 @@
         <v>34.700000000000003</v>
       </c>
     </row>
-    <row r="12" spans="1:46" ht="20" customHeight="1" x14ac:dyDescent="0.75">
+    <row r="12" spans="1:48" ht="20" customHeight="1" x14ac:dyDescent="0.75">
       <c r="A12" t="s">
         <v>9</v>
       </c>
@@ -12053,7 +12059,7 @@
         <v>37.4</v>
       </c>
     </row>
-    <row r="13" spans="1:46" ht="20" customHeight="1" x14ac:dyDescent="0.75">
+    <row r="13" spans="1:48" ht="20" customHeight="1" x14ac:dyDescent="0.75">
       <c r="A13" t="s">
         <v>9</v>
       </c>
@@ -12115,7 +12121,7 @@
         <v>20.2</v>
       </c>
     </row>
-    <row r="14" spans="1:46" ht="20" customHeight="1" x14ac:dyDescent="0.75">
+    <row r="14" spans="1:48" ht="20" customHeight="1" x14ac:dyDescent="0.75">
       <c r="A14" t="s">
         <v>9</v>
       </c>
@@ -12177,7 +12183,7 @@
         <v>26.8</v>
       </c>
     </row>
-    <row r="15" spans="1:46" ht="20" customHeight="1" x14ac:dyDescent="0.75">
+    <row r="15" spans="1:48" ht="20" customHeight="1" x14ac:dyDescent="0.75">
       <c r="A15" t="s">
         <v>9</v>
       </c>
@@ -12233,7 +12239,7 @@
         <v>6.8</v>
       </c>
     </row>
-    <row r="16" spans="1:46" ht="20" customHeight="1" x14ac:dyDescent="0.75">
+    <row r="16" spans="1:48" ht="20" customHeight="1" x14ac:dyDescent="0.75">
       <c r="A16" t="s">
         <v>9</v>
       </c>
@@ -16046,7 +16052,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="81" spans="1:46" ht="20" customHeight="1" x14ac:dyDescent="0.75">
+    <row r="81" spans="1:48" ht="20" customHeight="1" x14ac:dyDescent="0.75">
       <c r="A81" t="s">
         <v>849</v>
       </c>
@@ -16105,7 +16111,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="82" spans="1:46" ht="20" customHeight="1" x14ac:dyDescent="0.75">
+    <row r="82" spans="1:48" ht="20" customHeight="1" x14ac:dyDescent="0.75">
       <c r="A82" t="s">
         <v>849</v>
       </c>
@@ -16164,7 +16170,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="83" spans="1:46" ht="20" customHeight="1" x14ac:dyDescent="0.75">
+    <row r="83" spans="1:48" ht="20" customHeight="1" x14ac:dyDescent="0.75">
       <c r="A83" t="s">
         <v>849</v>
       </c>
@@ -16220,7 +16226,7 @@
         <v>306</v>
       </c>
     </row>
-    <row r="84" spans="1:46" ht="20" customHeight="1" x14ac:dyDescent="0.75">
+    <row r="84" spans="1:48" ht="20" customHeight="1" x14ac:dyDescent="0.75">
       <c r="A84" t="s">
         <v>849</v>
       </c>
@@ -16279,7 +16285,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="85" spans="1:46" ht="20" customHeight="1" x14ac:dyDescent="0.75">
+    <row r="85" spans="1:48" ht="20" customHeight="1" x14ac:dyDescent="0.75">
       <c r="A85" t="s">
         <v>849</v>
       </c>
@@ -16338,7 +16344,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="86" spans="1:46" ht="20" customHeight="1" x14ac:dyDescent="0.75">
+    <row r="86" spans="1:48" ht="20" customHeight="1" x14ac:dyDescent="0.75">
       <c r="A86" t="s">
         <v>849</v>
       </c>
@@ -16397,7 +16403,7 @@
         <v>3146</v>
       </c>
     </row>
-    <row r="87" spans="1:46" ht="20" customHeight="1" x14ac:dyDescent="0.75">
+    <row r="87" spans="1:48" ht="20" customHeight="1" x14ac:dyDescent="0.75">
       <c r="A87" t="s">
         <v>132</v>
       </c>
@@ -16462,7 +16468,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="88" spans="1:46" ht="20" customHeight="1" x14ac:dyDescent="0.75">
+    <row r="88" spans="1:48" ht="20" customHeight="1" x14ac:dyDescent="0.75">
       <c r="A88" t="s">
         <v>1085</v>
       </c>
@@ -16539,7 +16545,7 @@
         <v>4.97</v>
       </c>
     </row>
-    <row r="89" spans="1:46" ht="20" customHeight="1" x14ac:dyDescent="0.75">
+    <row r="89" spans="1:48" ht="20" customHeight="1" x14ac:dyDescent="0.75">
       <c r="A89" t="s">
         <v>134</v>
       </c>
@@ -16636,8 +16642,14 @@
       <c r="AT89">
         <v>26.6</v>
       </c>
-    </row>
-    <row r="90" spans="1:46" ht="20" customHeight="1" x14ac:dyDescent="0.75">
+      <c r="AU89">
+        <v>24.8</v>
+      </c>
+      <c r="AV89">
+        <v>22.6</v>
+      </c>
+    </row>
+    <row r="90" spans="1:48" ht="20" customHeight="1" x14ac:dyDescent="0.75">
       <c r="A90" t="s">
         <v>134</v>
       </c>
@@ -16731,11 +16743,17 @@
       <c r="AS90">
         <v>7.5</v>
       </c>
-      <c r="AT90">
+      <c r="AT90" s="7">
         <v>7</v>
       </c>
-    </row>
-    <row r="91" spans="1:46" ht="20" customHeight="1" x14ac:dyDescent="0.75">
+      <c r="AU90">
+        <v>7.1</v>
+      </c>
+      <c r="AV90">
+        <v>6.8</v>
+      </c>
+    </row>
+    <row r="91" spans="1:48" ht="20" customHeight="1" x14ac:dyDescent="0.75">
       <c r="A91" t="s">
         <v>134</v>
       </c>
@@ -16832,8 +16850,14 @@
       <c r="AT91">
         <v>4.7</v>
       </c>
-    </row>
-    <row r="92" spans="1:46" ht="20" customHeight="1" x14ac:dyDescent="0.75">
+      <c r="AU91" s="7">
+        <v>4</v>
+      </c>
+      <c r="AV91">
+        <v>3.6</v>
+      </c>
+    </row>
+    <row r="92" spans="1:48" ht="20" customHeight="1" x14ac:dyDescent="0.75">
       <c r="A92" t="s">
         <v>134</v>
       </c>
@@ -16930,8 +16954,14 @@
       <c r="AT92">
         <v>14.9</v>
       </c>
-    </row>
-    <row r="93" spans="1:46" ht="20" customHeight="1" x14ac:dyDescent="0.75">
+      <c r="AU92">
+        <v>13.7</v>
+      </c>
+      <c r="AV92">
+        <v>12.2</v>
+      </c>
+    </row>
+    <row r="93" spans="1:48" ht="20" customHeight="1" x14ac:dyDescent="0.75">
       <c r="A93" t="s">
         <v>135</v>
       </c>
@@ -16982,7 +17012,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="94" spans="1:46" ht="20" customHeight="1" x14ac:dyDescent="0.75">
+    <row r="94" spans="1:48" ht="20" customHeight="1" x14ac:dyDescent="0.75">
       <c r="A94" t="s">
         <v>135</v>
       </c>
@@ -17042,7 +17072,7 @@
         <v>17.2</v>
       </c>
     </row>
-    <row r="95" spans="1:46" ht="20" customHeight="1" x14ac:dyDescent="0.75">
+    <row r="95" spans="1:48" ht="20" customHeight="1" x14ac:dyDescent="0.75">
       <c r="A95" t="s">
         <v>135</v>
       </c>
@@ -17096,7 +17126,7 @@
         <v>19.2</v>
       </c>
     </row>
-    <row r="96" spans="1:46" ht="20" customHeight="1" x14ac:dyDescent="0.75">
+    <row r="96" spans="1:48" ht="20" customHeight="1" x14ac:dyDescent="0.75">
       <c r="A96" t="s">
         <v>843</v>
       </c>

</xml_diff>

<commit_message>
Make 2025 and 2026 updates possible; update DSD
</commit_message>
<xml_diff>
--- a/data/2025_RW-SDG_Data.xlsx
+++ b/data/2025_RW-SDG_Data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\GGessienne\Documents\sdg-data-rwanda\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{50C72346-FE13-423F-A1B3-986E79831C49}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C798CD4E-6556-4972-832D-C886FC700565}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-90" yWindow="-90" windowWidth="19380" windowHeight="10260" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-90" yWindow="-90" windowWidth="19380" windowHeight="10260" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Data" sheetId="1" r:id="rId1"/>
@@ -45572,7 +45572,7 @@
         <v>110</v>
       </c>
       <c r="G2" s="3">
-        <v>25</v>
+        <v>27</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.75">

</xml_diff>